<commit_message>
change order of sheets
</commit_message>
<xml_diff>
--- a/docs/resources/Dictionary_testCohort.xlsx
+++ b/docs/resources/Dictionary_testCohort.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HijmansBS\Molgenis\repos\molgenis-emx2\docs\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E20DF1E-57B5-4C45-8507-F958381E2CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487BF35E-9977-40B9-AAD9-971644DA6AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Variables" sheetId="13" r:id="rId1"/>
-    <sheet name="Tables" sheetId="9" r:id="rId2"/>
+    <sheet name="Tables" sheetId="9" r:id="rId1"/>
+    <sheet name="Variables" sheetId="13" r:id="rId2"/>
     <sheet name="Variable values" sheetId="20" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -824,6 +824,216 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:V20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1427,216 +1637,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>140</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" t="s">
-        <v>125</v>
-      </c>
-      <c r="E3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4" t="s">
-        <v>125</v>
-      </c>
-      <c r="E4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H4" t="s">
-        <v>51</v>
-      </c>
-      <c r="I4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" t="s">
-        <v>125</v>
-      </c>
-      <c r="E5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H5" t="s">
-        <v>55</v>
-      </c>
-      <c r="I5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" t="s">
-        <v>125</v>
-      </c>
-      <c r="E6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" t="s">
-        <v>59</v>
-      </c>
-      <c r="I6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" t="s">
-        <v>125</v>
-      </c>
-      <c r="E7" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" t="s">
-        <v>62</v>
-      </c>
-      <c r="H7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:J4"/>

</xml_diff>

<commit_message>
fix: change order of sheets (#6806)
</commit_message>
<xml_diff>
--- a/docs/resources/Dictionary_testCohort.xlsx
+++ b/docs/resources/Dictionary_testCohort.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HijmansBS\Molgenis\repos\molgenis-emx2\docs\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E20DF1E-57B5-4C45-8507-F958381E2CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487BF35E-9977-40B9-AAD9-971644DA6AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Variables" sheetId="13" r:id="rId1"/>
-    <sheet name="Tables" sheetId="9" r:id="rId2"/>
+    <sheet name="Tables" sheetId="9" r:id="rId1"/>
+    <sheet name="Variables" sheetId="13" r:id="rId2"/>
     <sheet name="Variable values" sheetId="20" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
@@ -824,6 +824,216 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" t="s">
+        <v>59</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" t="s">
+        <v>59</v>
+      </c>
+      <c r="I7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:V20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1427,216 +1637,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.21875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>140</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" t="s">
-        <v>41</v>
-      </c>
-      <c r="H2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" t="s">
-        <v>125</v>
-      </c>
-      <c r="E3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4" t="s">
-        <v>125</v>
-      </c>
-      <c r="E4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H4" t="s">
-        <v>51</v>
-      </c>
-      <c r="I4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" t="s">
-        <v>125</v>
-      </c>
-      <c r="E5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H5" t="s">
-        <v>55</v>
-      </c>
-      <c r="I5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" t="s">
-        <v>125</v>
-      </c>
-      <c r="E6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" t="s">
-        <v>58</v>
-      </c>
-      <c r="H6" t="s">
-        <v>59</v>
-      </c>
-      <c r="I6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" t="s">
-        <v>125</v>
-      </c>
-      <c r="E7" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" t="s">
-        <v>62</v>
-      </c>
-      <c r="H7" t="s">
-        <v>59</v>
-      </c>
-      <c r="I7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:J4"/>

</xml_diff>